<commit_message>
feat(glossary): counters as {name, group_id, group_name, large_group, feature_id} objects
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/spar/data/samples/counter_ref_sample.xlsx
+++ b/spar/data/samples/counter_ref_sample.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -489,6 +489,11 @@
           <t>Max</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Feature ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -536,11 +541,13 @@
           <t>1024</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>FGR-HO0101</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>CELL.UE.ActiveNbr</t>
@@ -571,11 +578,13 @@
           <t>1024</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>FGR-HO0101</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>CELL.UE.IdleNbr</t>
@@ -606,9 +615,13 @@
           <t>1024</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>FGR-HO0101</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n"/>
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>RRC Setup</t>
@@ -649,11 +662,13 @@
           <t>65535</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>FGR-RS0101</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
           <t>CELL.RRC.SetupSucc</t>
@@ -684,11 +699,13 @@
           <t>65535</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>FGR-RS0101</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="inlineStr">
         <is>
           <t>CELL.RRC.SetupFail</t>
@@ -717,6 +734,11 @@
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>65535</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>FGR-RS0101</t>
         </is>
       </c>
     </row>
@@ -766,11 +788,13 @@
           <t>100</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>FGR-BW0301</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
       <c r="D9" s="2" t="inlineStr">
         <is>
           <t>CELL.MAC.DlThroughput</t>
@@ -801,11 +825,13 @@
           <t>10000000</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>FGR-BW0301</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
           <t>CELL.MAC.DlRetxRatio</t>
@@ -836,9 +862,13 @@
           <t>100</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>FGR-BW0301</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
       <c r="B11" s="2" t="inlineStr">
         <is>
           <t>PUSCH</t>
@@ -879,11 +909,13 @@
           <t>100</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>FGR-BW0301</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
           <t>CELL.MAC.UlThroughput</t>
@@ -912,6 +944,11 @@
       <c r="I12" s="2" t="inlineStr">
         <is>
           <t>5000000</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>FGR-BW0301</t>
         </is>
       </c>
     </row>
@@ -961,11 +998,13 @@
           <t>-44</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>FGR-HO0102</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
           <t>CELL.PHY.AvgSINR</t>
@@ -994,6 +1033,11 @@
       <c r="I14" s="2" t="inlineStr">
         <is>
           <t>30</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>FGR-HO0102</t>
         </is>
       </c>
     </row>
@@ -1001,8 +1045,8 @@
   <mergeCells count="13">
     <mergeCell ref="A13:A14"/>
     <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A8:A12"/>
     <mergeCell ref="C2:C4"/>
-    <mergeCell ref="A8:A12"/>
     <mergeCell ref="A2:A7"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="C5:C7"/>

</xml_diff>